<commit_message>
Part III - ELECTRE 1s
</commit_message>
<xml_diff>
--- a/PROJEKT.xlsx
+++ b/PROJEKT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24701"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Studia\S5 - Wspomaganie Decyzji\Raport\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11274F06-7F34-4A5A-8F9E-91891144C1D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{347F2916-F1BD-4E88-8818-8D362E22329E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="22320" windowHeight="13176" xr2:uid="{C57944E7-ABCB-44C1-8BAA-AA3DEE6AAFB1}"/>
+    <workbookView xWindow="-4788" yWindow="3036" windowWidth="16584" windowHeight="9420" xr2:uid="{C57944E7-ABCB-44C1-8BAA-AA3DEE6AAFB1}"/>
   </bookViews>
   <sheets>
     <sheet name="CONCERT - PROGRAM" sheetId="1" r:id="rId1"/>
@@ -57,30 +57,6 @@
     <t>+</t>
   </si>
   <si>
-    <t>Muzyka pop</t>
-  </si>
-  <si>
-    <t>Monofoniczna muzyka filmowa / growa</t>
-  </si>
-  <si>
-    <t>Monofoniczna muzyka klasyczna</t>
-  </si>
-  <si>
-    <t>Polifoniczna muzyka filmowa / growa</t>
-  </si>
-  <si>
-    <t>Orkiestrowa polifoniczna muzyka filmowa / growa</t>
-  </si>
-  <si>
-    <t>Polifoniczna muzyka klasyczna</t>
-  </si>
-  <si>
-    <t>Orkiestrowa polifoniczna muzyka klasyczna</t>
-  </si>
-  <si>
-    <t>Muzyka musicalowa</t>
-  </si>
-  <si>
     <t>Czas wykonania +</t>
   </si>
   <si>
@@ -126,27 +102,6 @@
     <t>The Mission Suite (E. Morricone)</t>
   </si>
   <si>
-    <t>Kameralna</t>
-  </si>
-  <si>
-    <t>Mała</t>
-  </si>
-  <si>
-    <t>Średnia</t>
-  </si>
-  <si>
-    <t>Duża</t>
-  </si>
-  <si>
-    <t>Pełna</t>
-  </si>
-  <si>
-    <t>Filmowa</t>
-  </si>
-  <si>
-    <t>Solo</t>
-  </si>
-  <si>
     <t>Gatunek</t>
   </si>
   <si>
@@ -271,6 +226,51 @@
   </si>
   <si>
     <t>Liczba wyświetleń</t>
+  </si>
+  <si>
+    <t>Muzyka pop (1)</t>
+  </si>
+  <si>
+    <t>Polifoniczna muzyka filmowa / growa (4)</t>
+  </si>
+  <si>
+    <t>Monofoniczna muzyka filmowa / growa (2)</t>
+  </si>
+  <si>
+    <t>Monofoniczna muzyka klasyczna (3)</t>
+  </si>
+  <si>
+    <t>Orkiestrowa polifoniczna muzyka filmowa / growa (6)</t>
+  </si>
+  <si>
+    <t>Muzyka musicalowa (5)</t>
+  </si>
+  <si>
+    <t>Polifoniczna muzyka klasyczna (7)</t>
+  </si>
+  <si>
+    <t>Orkiestrowa polifoniczna muzyka klasyczna (8)</t>
+  </si>
+  <si>
+    <t>Solo (1)</t>
+  </si>
+  <si>
+    <t>Kameralna (2)</t>
+  </si>
+  <si>
+    <t>Mała (3)</t>
+  </si>
+  <si>
+    <t>Średnia (4)</t>
+  </si>
+  <si>
+    <t>Duża (5)</t>
+  </si>
+  <si>
+    <t>Pełna (6)</t>
+  </si>
+  <si>
+    <t>Filmowa (7)</t>
   </si>
 </sst>
 </file>
@@ -439,7 +439,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -469,13 +475,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -808,10 +808,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="D2" s="1" t="s">
@@ -838,34 +838,34 @@
         <v>3</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="H3" s="34" t="s">
-        <v>78</v>
+        <v>46</v>
+      </c>
+      <c r="H3" s="22" t="s">
+        <v>63</v>
       </c>
       <c r="I3" s="7" t="s">
         <v>6</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="32"/>
+      <c r="A4" s="23"/>
       <c r="B4" s="3">
         <v>1</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="E4" s="3">
         <v>10</v>
@@ -874,28 +874,28 @@
         <v>7</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="32"/>
+      <c r="A5" s="23"/>
       <c r="B5" s="3">
         <v>2</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>34</v>
+        <v>77</v>
       </c>
       <c r="E5" s="3">
         <v>10</v>
@@ -904,28 +904,28 @@
         <v>7</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>13</v>
+        <v>71</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="I5" s="7" t="s">
         <v>4</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="32"/>
+      <c r="A6" s="23"/>
       <c r="B6" s="3">
         <v>3</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>36</v>
+        <v>72</v>
       </c>
       <c r="E6" s="3">
         <v>6</v>
@@ -934,24 +934,24 @@
         <v>7</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="I6" s="5"/>
       <c r="J6" s="3"/>
     </row>
     <row r="7" spans="1:10" s="2" customFormat="1" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="32"/>
+      <c r="A7" s="23"/>
       <c r="B7" s="4">
         <v>4</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>36</v>
+        <v>72</v>
       </c>
       <c r="E7" s="4">
         <v>8.5</v>
@@ -960,24 +960,24 @@
         <v>8</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
     </row>
     <row r="8" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="32"/>
+      <c r="A8" s="23"/>
       <c r="B8" s="3">
         <v>5</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>32</v>
+        <v>75</v>
       </c>
       <c r="E8" s="3">
         <v>1</v>
@@ -986,24 +986,24 @@
         <v>7</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
     </row>
     <row r="9" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="32"/>
+      <c r="A9" s="23"/>
       <c r="B9" s="3">
         <v>6</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>36</v>
+        <v>72</v>
       </c>
       <c r="E9" s="3">
         <v>4</v>
@@ -1012,24 +1012,24 @@
         <v>1</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>10</v>
+        <v>65</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
     </row>
     <row r="10" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="32"/>
+      <c r="A10" s="23"/>
       <c r="B10" s="7">
         <v>7</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>34</v>
+        <v>77</v>
       </c>
       <c r="E10" s="3">
         <v>3</v>
@@ -1038,23 +1038,23 @@
         <v>7</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>13</v>
+        <v>71</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="I10" s="3"/>
     </row>
     <row r="11" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="32"/>
+      <c r="A11" s="23"/>
       <c r="B11" s="7">
         <v>8</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>32</v>
+        <v>75</v>
       </c>
       <c r="E11" s="3">
         <v>4.5</v>
@@ -1063,23 +1063,23 @@
         <v>7</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="I11" s="3"/>
     </row>
     <row r="12" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="32"/>
+      <c r="A12" s="23"/>
       <c r="B12" s="7">
         <v>9</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>30</v>
+        <v>73</v>
       </c>
       <c r="E12" s="3">
         <v>4</v>
@@ -1088,23 +1088,23 @@
         <v>7</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>7</v>
+        <v>64</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="I12" s="3"/>
     </row>
     <row r="13" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="32"/>
+      <c r="A13" s="23"/>
       <c r="B13" s="7">
         <v>10</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>31</v>
+        <v>74</v>
       </c>
       <c r="E13" s="3">
         <v>2.5</v>
@@ -1113,23 +1113,23 @@
         <v>7</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="I13" s="3"/>
     </row>
     <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="32"/>
+      <c r="A14" s="23"/>
       <c r="B14" s="7">
         <v>11</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>33</v>
+        <v>76</v>
       </c>
       <c r="E14" s="3">
         <v>4</v>
@@ -1138,23 +1138,23 @@
         <v>7</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>10</v>
+        <v>65</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="I14" s="3"/>
     </row>
     <row r="15" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="32"/>
+      <c r="A15" s="23"/>
       <c r="B15" s="7">
         <v>12</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="E15" s="3">
         <v>4</v>
@@ -1163,23 +1163,23 @@
         <v>6</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="I15" s="3"/>
     </row>
     <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="32"/>
+      <c r="A16" s="23"/>
       <c r="B16" s="7">
         <v>13</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>31</v>
+        <v>74</v>
       </c>
       <c r="E16" s="3">
         <v>6</v>
@@ -1188,23 +1188,23 @@
         <v>10</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>7</v>
+        <v>64</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="I16" s="3"/>
     </row>
     <row r="17" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A17" s="32"/>
+      <c r="A17" s="23"/>
       <c r="B17" s="7">
         <v>14</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>32</v>
+        <v>74</v>
       </c>
       <c r="E17" s="3">
         <v>0</v>
@@ -1213,23 +1213,23 @@
         <v>1</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>10</v>
+        <v>68</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="I17" s="3"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B20" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="C20" s="22"/>
+      <c r="B20" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" s="34"/>
       <c r="I20" s="6"/>
     </row>
     <row r="21" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>3</v>
@@ -1240,7 +1240,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>36</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
@@ -1248,7 +1248,7 @@
         <v>2</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>30</v>
+        <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
@@ -1256,7 +1256,7 @@
         <v>3</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>31</v>
+        <v>74</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
@@ -1264,7 +1264,7 @@
         <v>4</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>32</v>
+        <v>75</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
@@ -1272,7 +1272,7 @@
         <v>5</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>33</v>
+        <v>76</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
@@ -1280,7 +1280,7 @@
         <v>6</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>34</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
@@ -1288,21 +1288,21 @@
         <v>7</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B30" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="C30" s="22"/>
+      <c r="B30" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="C30" s="34"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
@@ -1310,7 +1310,7 @@
         <v>3</v>
       </c>
       <c r="C32" s="18" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.3">
@@ -1318,7 +1318,7 @@
         <v>4.5</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.3">
@@ -1326,7 +1326,7 @@
         <v>8.5</v>
       </c>
       <c r="C34" s="18" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.3">
@@ -1334,7 +1334,7 @@
         <v>10</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.3">
@@ -1342,21 +1342,21 @@
         <v>30</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B38" s="22" t="s">
-        <v>64</v>
-      </c>
-      <c r="C38" s="22"/>
+      <c r="B38" s="34" t="s">
+        <v>49</v>
+      </c>
+      <c r="C38" s="34"/>
     </row>
     <row r="39" spans="2:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B39" s="16" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="C39" s="17" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
     </row>
     <row r="40" spans="2:3" x14ac:dyDescent="0.3">
@@ -1364,7 +1364,7 @@
         <v>1</v>
       </c>
       <c r="C40" s="18" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.3">
@@ -1372,7 +1372,7 @@
         <v>2</v>
       </c>
       <c r="C41" s="19" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
     </row>
     <row r="42" spans="2:3" x14ac:dyDescent="0.3">
@@ -1380,7 +1380,7 @@
         <v>3</v>
       </c>
       <c r="C42" s="18" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
     </row>
     <row r="43" spans="2:3" x14ac:dyDescent="0.3">
@@ -1388,7 +1388,7 @@
         <v>4</v>
       </c>
       <c r="C43" s="19" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="44" spans="2:3" x14ac:dyDescent="0.3">
@@ -1396,7 +1396,7 @@
         <v>5</v>
       </c>
       <c r="C44" s="18" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
     </row>
     <row r="45" spans="2:3" x14ac:dyDescent="0.3">
@@ -1404,7 +1404,7 @@
         <v>6</v>
       </c>
       <c r="C45" s="19" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
     </row>
     <row r="46" spans="2:3" x14ac:dyDescent="0.3">
@@ -1412,7 +1412,7 @@
         <v>7</v>
       </c>
       <c r="C46" s="18" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.3">
@@ -1420,7 +1420,7 @@
         <v>8</v>
       </c>
       <c r="C47" s="19" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
     </row>
     <row r="48" spans="2:3" x14ac:dyDescent="0.3">
@@ -1428,7 +1428,7 @@
         <v>9</v>
       </c>
       <c r="C48" s="18" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.3">
@@ -1436,104 +1436,104 @@
         <v>10</v>
       </c>
       <c r="C49" s="15" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B51" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="C51" s="22"/>
+      <c r="B51" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="C51" s="34"/>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B52" t="s">
-        <v>49</v>
-      </c>
-      <c r="C52" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="D52" s="30"/>
-      <c r="E52" s="31"/>
+        <v>34</v>
+      </c>
+      <c r="C52" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="D52" s="32"/>
+      <c r="E52" s="33"/>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B53">
         <v>1</v>
       </c>
-      <c r="C53" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="D53" s="24"/>
-      <c r="E53" s="25"/>
+      <c r="C53" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53" s="26"/>
+      <c r="E53" s="27"/>
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B54">
         <v>2</v>
       </c>
-      <c r="C54" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="D54" s="27"/>
-      <c r="E54" s="28"/>
+      <c r="C54" s="28" t="s">
+        <v>66</v>
+      </c>
+      <c r="D54" s="29"/>
+      <c r="E54" s="30"/>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B55">
         <v>3</v>
       </c>
-      <c r="C55" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="D55" s="24"/>
-      <c r="E55" s="25"/>
+      <c r="C55" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="D55" s="26"/>
+      <c r="E55" s="27"/>
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B56">
         <v>4</v>
       </c>
-      <c r="C56" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="D56" s="27"/>
-      <c r="E56" s="28"/>
+      <c r="C56" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="D56" s="29"/>
+      <c r="E56" s="30"/>
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B57">
         <v>5</v>
       </c>
-      <c r="C57" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="D57" s="24"/>
-      <c r="E57" s="25"/>
+      <c r="C57" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="D57" s="26"/>
+      <c r="E57" s="27"/>
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B58">
         <v>6</v>
       </c>
-      <c r="C58" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="D58" s="27"/>
-      <c r="E58" s="28"/>
+      <c r="C58" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="D58" s="29"/>
+      <c r="E58" s="30"/>
     </row>
     <row r="59" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B59">
         <v>7</v>
       </c>
-      <c r="C59" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="D59" s="24"/>
-      <c r="E59" s="25"/>
+      <c r="C59" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="D59" s="26"/>
+      <c r="E59" s="27"/>
     </row>
     <row r="60" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B60">
         <v>8</v>
       </c>
-      <c r="C60" s="26" t="s">
-        <v>13</v>
-      </c>
-      <c r="D60" s="27"/>
-      <c r="E60" s="28"/>
+      <c r="C60" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="D60" s="29"/>
+      <c r="E60" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="15">

</xml_diff>